<commit_message>
feat: add name sign, summary
</commit_message>
<xml_diff>
--- a/backend/fixtures/sample-ioffice.xlsx
+++ b/backend/fixtures/sample-ioffice.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,9 +410,12 @@
         <v>Văn bản ký số</v>
       </c>
       <c r="D1" t="str">
+        <v>Người ký chính</v>
+      </c>
+      <c r="E1" t="str">
         <v>Ngày ban hành</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Đơn vị ban hành</v>
       </c>
     </row>
@@ -427,9 +430,12 @@
         <v>Đã ký số</v>
       </c>
       <c r="D2" t="str">
+        <v>Nguyễn Văn A</v>
+      </c>
+      <c r="E2" t="str">
         <v>01/08/2026</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>ALCO</v>
       </c>
     </row>
@@ -444,9 +450,12 @@
         <v>Đã ký số</v>
       </c>
       <c r="D3" t="str">
+        <v>Trần Thị B</v>
+      </c>
+      <c r="E3" t="str">
         <v>02/08/2026</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Ban Khách hàng doanh nghiệp</v>
       </c>
     </row>
@@ -461,9 +470,12 @@
         <v/>
       </c>
       <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
         <v>03/08/2026</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Chi nhánh mẫu</v>
       </c>
     </row>
@@ -478,9 +490,12 @@
         <v>Đã ký số</v>
       </c>
       <c r="D5" t="str">
+        <v>Lê Văn C</v>
+      </c>
+      <c r="E5" t="str">
         <v>04/08/2026</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>Chi nhánh mẫu</v>
       </c>
     </row>
@@ -495,9 +510,12 @@
         <v/>
       </c>
       <c r="D6" t="str">
+        <v>Phạm Thị D</v>
+      </c>
+      <c r="E6" t="str">
         <v>05/08/2026</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>Văn phòng Trụ sở chính</v>
       </c>
     </row>
@@ -512,9 +530,12 @@
         <v>Đã ký số</v>
       </c>
       <c r="D7" t="str">
+        <v>Hoàng Văn E</v>
+      </c>
+      <c r="E7" t="str">
         <v>06/08/2026</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>NHNo</v>
       </c>
     </row>
@@ -529,15 +550,18 @@
         <v>Đã ký số</v>
       </c>
       <c r="D8" t="str">
+        <v>Đỗ Thị F</v>
+      </c>
+      <c r="E8" t="str">
         <v>07/08/2026</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>Agribank</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>